<commit_message>
[progress] new way request
</commit_message>
<xml_diff>
--- a/inv_state.xlsx
+++ b/inv_state.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,112 +438,70 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>B0183-W14-2408280011</t>
+          <t>B0183-W11-2408290001</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>B0183-W11-2408280023</t>
+          <t>B0183-W11-2408290006</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>B0183-w12-2408280006</t>
+          <t>B0183-W11-2408290007</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>B0183-w12-2408280007</t>
+          <t>B0183-W11-2408290008</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B0183-w12-2408280008</t>
+          <t>B0183-W11-2408290009</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>B0183-w12-2408280009</t>
+          <t>B0183-W11-2408290010</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>B0183-W14-2408280014</t>
+          <t>B0183-W11-2408290011</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>B0183-W14-2408280023</t>
+          <t>B0183-W11-2408290012</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>B0183-W14-2408280029</t>
+          <t>B0183-W11-2408290013</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B0183-W14-2408280030</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>B0183-W14-2408280031</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>B0183-w12-2408280010</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>B0183-W14-2408280037</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>B0183-W14-2408280038</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>B0183-W14-2408280039</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>B0183-W14-2408280040</t>
+          <t>B0183-W11-2408290014</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[BugFixed] Start n stop btn
</commit_message>
<xml_diff>
--- a/inv_state.xlsx
+++ b/inv_state.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,39 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B0183-W04-2408280001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B0183-W35-2408280036</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B0183-W05-2408280047</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B0183-W35-2408280037</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B0183-W35-2408280038</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
[adjust] change display ui-log
</commit_message>
<xml_diff>
--- a/inv_state.xlsx
+++ b/inv_state.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,39 +436,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>B0183-W04-2408280001</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>B0183-W35-2408280036</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>B0183-W05-2408280047</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>B0183-W35-2408280037</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>B0183-W35-2408280038</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>